<commit_message>
research: Latent Reasoning에 RecursiveMAS (arXiv 2604.25917) 추가 - 2026-05-18
- RecursiveMAS: Multi-Agent System으로 Latent Reasoning을 확장
  (Inner/Outer RecursiveLink, Inner-Outer Loop 학습, 4가지 협업 패턴)
- 블로그: 7번 섹션 신설, 종합 지형도를 5가지 흐름으로 확장, 미해결 과제 갱신
- 슬라이드: RecursiveMAS 메커니즘/결과 슬라이드 2장 추가, 5가지 흐름 종합 슬라이드 갱신
- 참고문헌 XLSX: 논문/프로젝트 페이지/GitHub 3개 항목 추가
- index.md 홈페이지 항목을 2026-05-18 업데이트 표기로 변경

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/2026-05-08-latent-reasoning/latent-reasoning-references.xlsx
+++ b/2026-05-08-latent-reasoning/latent-reasoning-references.xlsx
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1125,6 +1125,111 @@
       <c r="G18" s="3" t="inlineStr">
         <is>
           <t>분류 체계 — Survey</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Recursive Multi-Agent Systems (RecursiveMAS)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Xiyuan Yang, Jiaru Zou, Rui Pan, Ruizhong Qiu, Pan Lu, Shizhe Diao, Jindong Jiang, Hanghang Tong, Tong Zhang, Markus J. Buehler, Jingrui He, James Zou / UIUC + Stanford + MIT + NVIDIA</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>https://arxiv.org/abs/2604.25917</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>Latent reasoning을 single model에서 multi-agent system으로 확장. RecursiveLink(Inner/Outer) 모듈로 agent 내부 latent feedback과 cross-agent latent state transfer 구현. Inner-Outer Loop 학습으로 RecursiveLink만 ~13M(0.31%) 학습. 9개 벤치마크(수학·과학·의학·검색·코드)에서 평균 +8.3%, 1.2-2.4x 가속, 34.6-75.6% 토큰 감소. Sequential/Mixture/Distillation/Deliberation 4가지 협업 패턴 검증. Theorem 4.1: latent recursion이 text recursion보다 gradient 안정성 증명.</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS 프로젝트 페이지</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Recursive Multi-Agent Systems Team</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>https://recursivemas.github.io</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS 공식 프로젝트 페이지. 아키텍처 다이어그램, 성능 결과, 코드/모델 링크 제공.</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS GitHub Repository</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS Team</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>https://github.com/RecursiveMAS/RecursiveMAS</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS 공식 코드 저장소. RecursiveLink 구현, 4가지 협업 패턴(Sequential/Mixture/Distillation/Deliberation) 학습 스크립트, HuggingFace 체크포인트 포함.</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>RecursiveMAS</t>
         </is>
       </c>
     </row>

</xml_diff>